<commit_message>
feat: implement chess scheduling engine backend, ingestion pipeline, and React frontend views
</commit_message>
<xml_diff>
--- a/backend/sample_data/mighty_knight_template.xlsx
+++ b/backend/sample_data/mighty_knight_template.xlsx
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Beginner 3</t>
+          <t>Beginner 2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Intermediate 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Basic 1, Basic 2, Beginner 1, Beginner 2, Beginner 3, Early Intermediate 1</t>
+          <t>Basic 1, Basic 2, Beginner 1, Beginner 2, Early Intermediate 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Beginner 1, Beginner 2, Beginner 3, Early Intermediate 1, Early Intermediate 2, Intermediate</t>
+          <t>Beginner 1, Beginner 2, Early Intermediate 1, Early Intermediate 2, Intermediate 1, Intermediate 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Early Intermediate 2, Intermediate</t>
+          <t>Early Intermediate 2, Intermediate 1, Intermediate 2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Beginner 2, Beginner 3, Early Intermediate 1, Intermediate</t>
+          <t>Beginner 2, Early Intermediate 1, Intermediate 1, Intermediate 2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Basic 1, Basic 2, Beginner 1, Beginner 2, Beginner 3, Early Intermediate 1, Early Intermediate 2, Intermediate</t>
+          <t>Basic 1, Basic 2, Beginner 1, Beginner 2, Early Intermediate 1, Early Intermediate 2, Intermediate 1, Intermediate 2, Advanced</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement rule engine, schedule services, and UI components
- Add baseline, effective schedule, master data, rule, and suggestion engines
- Add AbsoluteScheduleView, CompensationBadge, and RuleViolationModal components
- Update master data management, batch scheduling, daily planner, and settings views
- Update backend models, parsers, and test suites
</commit_message>
<xml_diff>
--- a/backend/sample_data/mighty_knight_template.xlsx
+++ b/backend/sample_data/mighty_knight_template.xlsx
@@ -1791,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1869,7 +1869,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Guruvanthana</t>
+          <t>GURU</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1923,7 +1923,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dhaanush</t>
+          <t>DHAANUSH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1977,7 +1977,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Arshath</t>
+          <t>ARSHATH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2031,7 +2031,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Saravanan</t>
+          <t>SARAVANAN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2085,7 +2085,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bathrinath</t>
+          <t>BATHRI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2139,7 +2139,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Abinaya</t>
+          <t>ABINAYA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2193,7 +2193,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Prakash</t>
+          <t>PRAKASH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2247,7 +2247,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Manikandan</t>
+          <t>MANIKANDAN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2297,6 +2297,60 @@
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HEMA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Basic 1, Basic 2, Beginner 1, Beginner 2, Tournament</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>20 - 40</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Evening</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Tournament only</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>